<commit_message>
Creating test cases and veryfing by asserting and finalizing the test cases
</commit_message>
<xml_diff>
--- a/src/test/resources/Test_Data/Sample_Execution.xlsx
+++ b/src/test/resources/Test_Data/Sample_Execution.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="18">
   <si>
     <t>UserName</t>
   </si>
@@ -80,6 +80,9 @@
   <si>
     <t>PASSED</t>
   </si>
+  <si>
+    <t>FAILED</t>
+  </si>
 </sst>
 </file>
 
@@ -251,7 +254,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -458,6 +461,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="42"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="10"/>
       </patternFill>
     </fill>
   </fills>
@@ -717,7 +730,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -727,6 +740,72 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
@@ -1314,7 +1393,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
     <col min="2" max="2" customWidth="true" width="15.0"/>
@@ -1356,6 +1435,336 @@
         <v>16</v>
       </c>
     </row>
+    <row r="3">
+      <c r="E3" t="s" s="6">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="E4" t="s" s="7">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="E5" t="s" s="8">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="E6" t="s" s="9">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="E7" t="s" s="10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="E8" t="s" s="11">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="E9" t="s" s="12">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="E10" t="s" s="13">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="E11" t="s" s="14">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="E12" t="s" s="15">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="E13" t="s" s="16">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" t="s" s="17">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" t="s" s="18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" t="s" s="19">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" t="s" s="20">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="E18" t="s" s="21">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="E19" t="s" s="22">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="E20" t="s" s="23">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" t="s" s="24">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" t="s" s="25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="E23" t="s" s="26">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="E24" t="s" s="27">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" t="s" s="28">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" t="s" s="29">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="E27" t="s" s="30">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" t="s" s="31">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="E29" t="s" s="32">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="E30" t="s" s="33">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" t="s" s="34">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" t="s" s="35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="E33" t="s" s="36">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34" t="s" s="37">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" t="s" s="38">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" t="s" s="39">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" t="s" s="40">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" t="s" s="41">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" t="s" s="42">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" t="s" s="43">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" t="s" s="44">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="E42" t="s" s="45">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="E43" t="s" s="46">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="E44" t="s" s="47">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="E45" t="s" s="48">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="E46" t="s" s="49">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="E47" t="s" s="50">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="E48" t="s" s="51">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="E49" t="s" s="52">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="E50" t="s" s="53">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="E51" t="s" s="54">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="E52" t="s" s="55">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="E53" t="s" s="56">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="E54" t="s" s="57">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="E55" t="s" s="58">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="E56" t="s" s="59">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="E57" t="s" s="60">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="E58" t="s" s="61">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="E59" t="s" s="62">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="E60" t="s" s="63">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="E61" t="s" s="64">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="E62" t="s" s="65">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="E63" t="s" s="66">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="E64" t="s" s="67">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="E65" t="s" s="68">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="E66" t="s" s="69">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="E67" t="s" s="70">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="E68" t="s" s="71">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>